<commit_message>
Added code for creating a plot of abundance index per field of every species in the Screening_Birds script
</commit_message>
<xml_diff>
--- a/data/original/Yield.xlsx
+++ b/data/original/Yield.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://irtacat-my.sharepoint.com/personal/alejandro_munoz_irta_cat/Documents/Documentos/Exclusion-Lisso-Analysis/data/original/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="103" documentId="8_{8B4FA26A-D4F7-4443-8C75-268ADA32ED06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{719350AC-7DFB-4A3F-A54F-F71032684C71}"/>
+  <xr:revisionPtr revIDLastSave="106" documentId="8_{8B4FA26A-D4F7-4443-8C75-268ADA32ED06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{714AD45B-9C78-40B6-AF08-8F406716B4E1}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-7515" windowWidth="29040" windowHeight="15720" xr2:uid="{4378E4F5-4D9E-4DF0-A2EC-28E161754BEC}"/>
   </bookViews>
@@ -95,7 +95,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000000"/>
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -151,37 +151,12 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="15">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -467,6 +442,31 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -511,44 +511,53 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DBEDB29B-7880-479C-B5C8-821ED7E21F63}" name="Tabla25" displayName="Tabla25" ref="A1:M81" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
-  <autoFilter ref="A1:M81" xr:uid="{DBEDB29B-7880-479C-B5C8-821ED7E21F63}"/>
+  <autoFilter ref="A1:M81" xr:uid="{DBEDB29B-7880-479C-B5C8-821ED7E21F63}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="4"/>
+        <filter val="5"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="2">
+      <filters>
+        <filter val="BE"/>
+        <filter val="FO"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{F4F9AD34-2BD1-4230-A1B9-807DA127C678}" name="Date" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{0D29DA5C-6A87-4734-B044-FA9437B84747}" name="Field" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{D97E7405-7B38-44FA-B9C3-73BF7396C810}" name="Treatment" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{B1967649-6994-481B-A304-9F8F097F3A38}" name="Repeat" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{89AD42B2-6B88-46F1-AB15-51ED923EAAF2}" name="Area_m2" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{C5755088-DA07-4DEC-89D7-7C30F8CE16AD}" name="Weight_g" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{8DE7F511-84B7-4EB5-BE31-FB6F570F165A}" name="Humidity" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{1573BD29-F3C8-4824-AF01-3B3473B33C0A}" name="Density" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{A73B6165-6ED4-4EBE-8F42-9B65F03EC49C}" name="Weight_kg/ha" dataDxfId="5">
+    <tableColumn id="1" xr3:uid="{F4F9AD34-2BD1-4230-A1B9-807DA127C678}" name="Date" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{0D29DA5C-6A87-4734-B044-FA9437B84747}" name="Field" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{D97E7405-7B38-44FA-B9C3-73BF7396C810}" name="Treatment" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{B1967649-6994-481B-A304-9F8F097F3A38}" name="Repeat" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{89AD42B2-6B88-46F1-AB15-51ED923EAAF2}" name="Area_m2" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{C5755088-DA07-4DEC-89D7-7C30F8CE16AD}" name="Weight_g" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{8DE7F511-84B7-4EB5-BE31-FB6F570F165A}" name="Humidity" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{1573BD29-F3C8-4824-AF01-3B3473B33C0A}" name="Density" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{A73B6165-6ED4-4EBE-8F42-9B65F03EC49C}" name="Weight_kg/ha" dataDxfId="4">
       <calculatedColumnFormula>Tabla25[[#This Row],[Weight_g]]*10000/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{3C40A40F-F087-4377-B13E-371FD648DF06}" name="Weight_reduction_prop" dataDxfId="4">
+    <tableColumn id="11" xr3:uid="{3C40A40F-F087-4377-B13E-371FD648DF06}" name="Weight_reduction_prop" dataDxfId="3">
       <calculatedColumnFormula>100*(Tabla25[[#This Row],[Humidity]]-14)/(100-Tabla25[[#This Row],[Humidity]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{DCD40F4E-7530-4353-BF5D-EB0A9C93E003}" name="Weight_reduction" dataDxfId="3">
+    <tableColumn id="12" xr3:uid="{DCD40F4E-7530-4353-BF5D-EB0A9C93E003}" name="Weight_reduction" dataDxfId="2">
       <calculatedColumnFormula>Tabla25[[#This Row],[Weight_kg/ha]]*Tabla25[[#This Row],[Weight_reduction_prop]]/100</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{499B7B4E-0029-46A3-945D-24DECC6672C5}" name="Yield_kg/ha_HR14" dataDxfId="2">
+    <tableColumn id="13" xr3:uid="{499B7B4E-0029-46A3-945D-24DECC6672C5}" name="Yield_kg/ha_HR14" dataDxfId="1">
       <calculatedColumnFormula>Tabla25[[#This Row],[Weight_kg/ha]]-Tabla25[[#This Row],[Weight_reduction]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3883EE77-DFF2-429D-BB67-CFA3BB8D147F}" name="Observations" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{3883EE77-DFF2-429D-BB67-CFA3BB8D147F}" name="Observations" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -586,7 +595,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -692,7 +701,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -834,7 +843,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -901,7 +910,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
         <v>45918</v>
       </c>
@@ -943,7 +952,7 @@
         <v>8263.7989540964554</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
         <v>45918</v>
       </c>
@@ -985,7 +994,7 @@
         <v>8156.314556739665</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
         <v>45918</v>
       </c>
@@ -1027,7 +1036,7 @@
         <v>9035.8818192670406</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>45918</v>
       </c>
@@ -1069,7 +1078,7 @@
         <v>8666.0463768115951</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>45918</v>
       </c>
@@ -1111,7 +1120,7 @@
         <v>7798.9218891916444</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>45918</v>
       </c>
@@ -1153,7 +1162,7 @@
         <v>8329.4026532807457</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>45918</v>
       </c>
@@ -1195,7 +1204,7 @@
         <v>8532.961832061068</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>45918</v>
       </c>
@@ -1237,7 +1246,7 @@
         <v>9188.2872266698541</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>45918</v>
       </c>
@@ -1279,7 +1288,7 @@
         <v>9116.1025641025644</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>45918</v>
       </c>
@@ -1321,7 +1330,7 @@
         <v>9453.264159923845</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>45918</v>
       </c>
@@ -1363,7 +1372,7 @@
         <v>9636.2436993100109</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>45918</v>
       </c>
@@ -1405,7 +1414,7 @@
         <v>9274.9172422149531</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>45918</v>
       </c>
@@ -1447,7 +1456,7 @@
         <v>9201.7444243520185</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>45918</v>
       </c>
@@ -1489,7 +1498,7 @@
         <v>9204.9712051190909</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>45918</v>
       </c>
@@ -1531,7 +1540,7 @@
         <v>9305.8038880986242</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>45918</v>
       </c>
@@ -1573,7 +1582,7 @@
         <v>8580.6185567010307</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>45918</v>
       </c>
@@ -1615,7 +1624,7 @@
         <v>10541.891713634728</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>45918</v>
       </c>
@@ -1657,7 +1666,7 @@
         <v>10320.531541348832</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>45918</v>
       </c>
@@ -1699,7 +1708,7 @@
         <v>9252.9069069069064</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>45918</v>
       </c>
@@ -1741,7 +1750,7 @@
         <v>10339.204208620884</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>45918</v>
       </c>
@@ -1783,7 +1792,7 @@
         <v>8560.9665071770341</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>45918</v>
       </c>
@@ -1825,7 +1834,7 @@
         <v>8789.7741383524808</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>45918</v>
       </c>
@@ -1867,7 +1876,7 @@
         <v>10125.214152700186</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>45918</v>
       </c>
@@ -1909,7 +1918,7 @@
         <v>8748.8627639155475</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>45918</v>
       </c>
@@ -1951,7 +1960,7 @@
         <v>8288.4742268041246</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>45918</v>
       </c>
@@ -1993,7 +2002,7 @@
         <v>8694.7118644067796</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>45918</v>
       </c>
@@ -2035,7 +2044,7 @@
         <v>9251.1015625</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>45918</v>
       </c>
@@ -2077,7 +2086,7 @@
         <v>8033.4520950747365</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>45918</v>
       </c>
@@ -2119,7 +2128,7 @@
         <v>8644.8338226658834</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>45918</v>
       </c>
@@ -2161,7 +2170,7 @@
         <v>9540.5717047239341</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>45918</v>
       </c>
@@ -2203,7 +2212,7 @@
         <v>9475.0743382086312</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>45918</v>
       </c>
@@ -2245,7 +2254,7 @@
         <v>9395.2402048350596</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>45917</v>
       </c>
@@ -2287,7 +2296,7 @@
         <v>8454.6643973601949</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
         <v>45917</v>
       </c>
@@ -2329,7 +2338,7 @@
         <v>8512.2326397593388</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
         <v>45917</v>
       </c>
@@ -2371,7 +2380,7 @@
         <v>8400.6121429454688</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="5">
         <v>45917</v>
       </c>
@@ -2413,7 +2422,7 @@
         <v>9140.2146565644034</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="5">
         <v>45917</v>
       </c>
@@ -2455,7 +2464,7 @@
         <v>7884.1749576168559</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="5">
         <v>45917</v>
       </c>
@@ -2497,7 +2506,7 @@
         <v>8798.2906044433421</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="5">
         <v>45917</v>
       </c>
@@ -2539,7 +2548,7 @@
         <v>9109.1807754817728</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="5">
         <v>45917</v>
       </c>
@@ -2581,7 +2590,7 @@
         <v>9310.6454330806519</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="5">
         <v>45917</v>
       </c>
@@ -2623,7 +2632,7 @@
         <v>8994.43976781524</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="5">
         <v>45917</v>
       </c>
@@ -2665,7 +2674,7 @@
         <v>9539.4810810810795</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="5">
         <v>45917</v>
       </c>
@@ -2707,7 +2716,7 @@
         <v>9168.5120611063212</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="5">
         <v>45917</v>
       </c>
@@ -2749,7 +2758,7 @@
         <v>8334.7218443664533</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="5">
         <v>45917</v>
       </c>
@@ -2791,7 +2800,7 @@
         <v>7318.0382128587007</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="5">
         <v>45917</v>
       </c>
@@ -2833,7 +2842,7 @@
         <v>8450.1588080831152</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="5">
         <v>45917</v>
       </c>
@@ -2875,7 +2884,7 @@
         <v>10142.278917378917</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="5">
         <v>45917</v>
       </c>
@@ -3085,7 +3094,7 @@
         <v>8651.0377336584243</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="5">
         <v>45919</v>
       </c>
@@ -3127,7 +3136,7 @@
         <v>6763.1981351981349</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="5">
         <v>45919</v>
       </c>
@@ -3169,7 +3178,7 @@
         <v>8406.2667899664775</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="5">
         <v>45919</v>
       </c>
@@ -3211,7 +3220,7 @@
         <v>7655.9134338666972</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="5">
         <v>45919</v>
       </c>
@@ -3421,7 +3430,7 @@
         <v>7127.8173454504658</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="5">
         <v>45919</v>
       </c>
@@ -3463,7 +3472,7 @@
         <v>7843.4911835887979</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="5">
         <v>45919</v>
       </c>
@@ -3505,7 +3514,7 @@
         <v>8513.6442465432392</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="5">
         <v>45919</v>
       </c>
@@ -3547,7 +3556,7 @@
         <v>6174.5649512582186</v>
       </c>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="5">
         <v>45919</v>
       </c>
@@ -3757,7 +3766,7 @@
         <v>9071.2530565167253</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="5">
         <v>45919</v>
       </c>
@@ -3799,7 +3808,7 @@
         <v>6514.6789092932668</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="5">
         <v>45919</v>
       </c>
@@ -3841,7 +3850,7 @@
         <v>10809.761673956733</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="5">
         <v>45919</v>
       </c>
@@ -3883,7 +3892,7 @@
         <v>8780.4588619402984</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="5">
         <v>45919</v>
       </c>
@@ -3925,7 +3934,7 @@
         <v>6758.4275412886718</v>
       </c>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="5">
         <v>45919</v>
       </c>
@@ -3967,7 +3976,7 @@
         <v>7739.2773397326018</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="5">
         <v>45919</v>
       </c>
@@ -4009,7 +4018,7 @@
         <v>9061.3228455754761</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="5">
         <v>45919</v>
       </c>
@@ -4051,7 +4060,7 @@
         <v>9791.4797367509527</v>
       </c>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="5">
         <v>45919</v>
       </c>

</xml_diff>